<commit_message>
feat: update dashboard formulas, receptionist shift guard, and incident classification
</commit_message>
<xml_diff>
--- a/homestayManagement/exports/temporary-residence/temporary-residence-2026-08-29.xlsx
+++ b/homestayManagement/exports/temporary-residence/temporary-residence-2026-08-29.xlsx
@@ -12,7 +12,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="31" uniqueCount="27">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="43" uniqueCount="31">
   <si>
     <t>DANH SÁCH KHAI BÁO TẠM TRÚ</t>
   </si>
@@ -53,46 +53,58 @@
     <t>Check-out dự kiến</t>
   </si>
   <si>
-    <t>BK_28082026_4</t>
+    <t>BK_29082026_4</t>
+  </si>
+  <si>
+    <t>102</t>
+  </si>
+  <si>
+    <t>Kỳ Anh Hoàng</t>
+  </si>
+  <si>
+    <t>0987654324</t>
+  </si>
+  <si>
+    <t>098765457523</t>
+  </si>
+  <si>
+    <t>Chí Linh Hải Dương</t>
   </si>
   <si>
     <t>101</t>
   </si>
   <si>
-    <t>Test</t>
-  </si>
-  <si>
-    <t>0968311853</t>
-  </si>
-  <si>
-    <t>026204007963</t>
-  </si>
-  <si>
-    <t>FPT</t>
-  </si>
-  <si>
-    <t>BK_29082026_1</t>
-  </si>
-  <si>
-    <t>quy</t>
-  </si>
-  <si>
-    <t>0989149456</t>
-  </si>
-  <si>
-    <t>026204007741</t>
-  </si>
-  <si>
-    <t>BK_29082026_3</t>
-  </si>
-  <si>
-    <t>Quý Quý</t>
-  </si>
-  <si>
-    <t>026204007965</t>
-  </si>
-  <si>
-    <t>Ha Noi</t>
+    <t>0987654323</t>
+  </si>
+  <si>
+    <t>098765464646</t>
+  </si>
+  <si>
+    <t>BK_29082026_7</t>
+  </si>
+  <si>
+    <t>0924998555</t>
+  </si>
+  <si>
+    <t>030087654321</t>
+  </si>
+  <si>
+    <t>BK_29082026_8</t>
+  </si>
+  <si>
+    <t>Nguyen Van An</t>
+  </si>
+  <si>
+    <t>0900000001</t>
+  </si>
+  <si>
+    <t>030205142423</t>
+  </si>
+  <si>
+    <t>Quan 1, TP Ho Chi Minh</t>
+  </si>
+  <si>
+    <t>BK_29082026_9</t>
   </si>
 </sst>
 </file>
@@ -206,13 +218,13 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <dimension ref="A1:K7"/>
+  <dimension ref="A1:K9"/>
   <sheetFormatPr defaultRowHeight="15.0"/>
   <cols>
     <col min="1" max="1" width="13.671875" customWidth="true" bestFit="true"/>
     <col min="2" max="2" width="17.1171875" customWidth="true" bestFit="true"/>
     <col min="3" max="3" width="13.671875" customWidth="true" bestFit="true"/>
-    <col min="4" max="4" width="13.671875" customWidth="true" bestFit="true"/>
+    <col min="4" max="4" width="16.37890625" customWidth="true" bestFit="true"/>
     <col min="5" max="5" width="13.671875" customWidth="true" bestFit="true"/>
     <col min="6" max="6" width="13.671875" customWidth="true" bestFit="true"/>
     <col min="7" max="7" width="14.87890625" customWidth="true" bestFit="true"/>
@@ -281,10 +293,10 @@
         <v>15</v>
       </c>
       <c r="E5" t="n" s="6">
-        <v>36621.0</v>
+        <v>38406.0</v>
       </c>
       <c r="F5" t="n" s="5">
-        <v>26.0</v>
+        <v>21.0</v>
       </c>
       <c r="G5" t="s" s="4">
         <v>16</v>
@@ -296,10 +308,10 @@
         <v>18</v>
       </c>
       <c r="J5" t="n" s="7">
-        <v>46263.04006608796</v>
+        <v>46263.672301666666</v>
       </c>
       <c r="K5" t="n" s="7">
-        <v>46263.041666666664</v>
+        <v>46263.75</v>
       </c>
     </row>
     <row r="6">
@@ -307,34 +319,34 @@
         <v>2.0</v>
       </c>
       <c r="B6" t="s" s="4">
+        <v>13</v>
+      </c>
+      <c r="C6" t="s" s="5">
         <v>19</v>
       </c>
-      <c r="C6" t="s" s="5">
-        <v>14</v>
-      </c>
       <c r="D6" t="s" s="4">
+        <v>15</v>
+      </c>
+      <c r="E6" t="n" s="6">
+        <v>38406.0</v>
+      </c>
+      <c r="F6" t="n" s="5">
+        <v>21.0</v>
+      </c>
+      <c r="G6" t="s" s="4">
         <v>20</v>
       </c>
-      <c r="E6" t="n" s="6">
-        <v>36621.0</v>
-      </c>
-      <c r="F6" t="n" s="5">
-        <v>26.0</v>
-      </c>
-      <c r="G6" t="s" s="4">
+      <c r="H6" t="s" s="4">
         <v>21</v>
-      </c>
-      <c r="H6" t="s" s="4">
-        <v>22</v>
       </c>
       <c r="I6" t="s" s="4">
         <v>18</v>
       </c>
       <c r="J6" t="n" s="7">
-        <v>46263.05271</v>
+        <v>46263.68264020833</v>
       </c>
       <c r="K6" t="n" s="7">
-        <v>46263.625</v>
+        <v>46263.75</v>
       </c>
     </row>
     <row r="7">
@@ -342,34 +354,104 @@
         <v>3.0</v>
       </c>
       <c r="B7" t="s" s="4">
-        <v>23</v>
+        <v>22</v>
       </c>
       <c r="C7" t="s" s="5">
         <v>14</v>
       </c>
       <c r="D7" t="s" s="4">
+        <v>15</v>
+      </c>
+      <c r="E7" t="n" s="6">
+        <v>38406.0</v>
+      </c>
+      <c r="F7" t="n" s="5">
+        <v>21.0</v>
+      </c>
+      <c r="G7" t="s" s="4">
+        <v>23</v>
+      </c>
+      <c r="H7" t="s" s="4">
         <v>24</v>
       </c>
-      <c r="E7" t="n" s="6">
-        <v>36621.0</v>
-      </c>
-      <c r="F7" t="n" s="5">
-        <v>26.0</v>
-      </c>
-      <c r="G7" t="s" s="4">
-        <v>16</v>
-      </c>
-      <c r="H7" t="s" s="4">
+      <c r="I7" t="s" s="4">
+        <v>18</v>
+      </c>
+      <c r="J7" t="n" s="7">
+        <v>46263.730481666666</v>
+      </c>
+      <c r="K7" t="n" s="7">
+        <v>46263.791666666664</v>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" t="n" s="5">
+        <v>4.0</v>
+      </c>
+      <c r="B8" t="s" s="4">
         <v>25</v>
       </c>
-      <c r="I7" t="s" s="4">
+      <c r="C8" t="s" s="5">
+        <v>14</v>
+      </c>
+      <c r="D8" t="s" s="4">
         <v>26</v>
       </c>
-      <c r="J7" t="n" s="7">
-        <v>46263.61499340278</v>
-      </c>
-      <c r="K7" t="n" s="7">
-        <v>46263.708333333336</v>
+      <c r="E8" t="n" s="6">
+        <v>34773.0</v>
+      </c>
+      <c r="F8" t="n" s="5">
+        <v>31.0</v>
+      </c>
+      <c r="G8" t="s" s="4">
+        <v>27</v>
+      </c>
+      <c r="H8" t="s" s="4">
+        <v>28</v>
+      </c>
+      <c r="I8" t="s" s="4">
+        <v>29</v>
+      </c>
+      <c r="J8" t="n" s="7">
+        <v>46263.73974460648</v>
+      </c>
+      <c r="K8" t="n" s="7">
+        <v>46263.833333333336</v>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" t="n" s="5">
+        <v>5.0</v>
+      </c>
+      <c r="B9" t="s" s="4">
+        <v>30</v>
+      </c>
+      <c r="C9" t="s" s="5">
+        <v>14</v>
+      </c>
+      <c r="D9" t="s" s="4">
+        <v>26</v>
+      </c>
+      <c r="E9" t="n" s="6">
+        <v>34773.0</v>
+      </c>
+      <c r="F9" t="n" s="5">
+        <v>31.0</v>
+      </c>
+      <c r="G9" t="s" s="4">
+        <v>27</v>
+      </c>
+      <c r="H9" t="s" s="4">
+        <v>28</v>
+      </c>
+      <c r="I9" t="s" s="4">
+        <v>29</v>
+      </c>
+      <c r="J9" t="n" s="7">
+        <v>46263.741088993054</v>
+      </c>
+      <c r="K9" t="n" s="7">
+        <v>46263.833333333336</v>
       </c>
     </row>
   </sheetData>

</xml_diff>